<commit_message>
Fix demo: 15/15 PASS — flexible parser + corrected sample data
- _utils.py: find_tfl_value now checks col-0 labels (AE summary layout)
  in addition to col-1 (demographics layout), enabling T-03 to match
- T14.3.1_AE_summary.docx: correct Drug A drug-related count (12→11)
- L16.2.7.2_SAE_listing.docx: add 3 missing SAE subjects (8 total)
- adsl.csv: add DTHFL column; 4 subjects flagged for deaths listing
- L16.2.7.3_deaths_listing.docx: use real ADSL subject IDs
- adrs.csv: new — 40 individual response records (ITT population)
- adpd.csv: new — 6 protocol deviation records
- L16.2.7.5_protocol_deviations.docx: use real ADSL subject IDs
- study_config.xlsx: L-03 listing_filter=DTHFL=='Y'; L-04→adrs.csv;
  L-05→adpd.csv; Datasets sheet updated with ADRS/ADPD entries
</commit_message>
<xml_diff>
--- a/study_config.xlsx
+++ b/study_config.xlsx
@@ -267,7 +267,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -348,6 +348,50 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -359,7 +403,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -570,6 +614,8 @@
     <xf numFmtId="0" fontId="18" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1298,7 +1344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="32" min="1" max="1"/>
@@ -2220,7 +2266,11 @@
           <t>SAFFL == 'Y'</t>
         </is>
       </c>
-      <c r="K16" s="47" t="n"/>
+      <c r="K16" s="47" t="inlineStr">
+        <is>
+          <t>DTHFL == 'Y'</t>
+        </is>
+      </c>
       <c r="L16" s="47" t="inlineStr">
         <is>
           <t>TRT01A</t>
@@ -2271,7 +2321,7 @@
       </c>
       <c r="G17" s="48" t="inlineStr">
         <is>
-          <t>adtte.csv</t>
+          <t>adrs.csv</t>
         </is>
       </c>
       <c r="H17" s="48" t="n"/>
@@ -2327,12 +2377,12 @@
       </c>
       <c r="F18" s="47" t="inlineStr">
         <is>
-          <t>ADSL</t>
+          <t>ADPD</t>
         </is>
       </c>
       <c r="G18" s="47" t="inlineStr">
         <is>
-          <t>adsl.csv</t>
+          <t>adpd.csv</t>
         </is>
       </c>
       <c r="H18" s="47" t="n"/>
@@ -2472,7 +2522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="32" min="1" max="1"/>
@@ -2665,7 +2715,7 @@
       </c>
       <c r="B9" s="59" t="inlineStr">
         <is>
-          <t>adtte.csv</t>
+          <t>adrs.csv</t>
         </is>
       </c>
       <c r="C9" s="59" t="inlineStr">
@@ -2681,6 +2731,33 @@
       <c r="E9" s="59" t="inlineStr">
         <is>
           <t>Response dataset (using ADTTE file for demo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ADPD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>adpd.csv</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ADaM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>USUBJID, TRT01A, PDCAT, PDTERM, SAFFL</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Protocol deviations dataset</t>
         </is>
       </c>
     </row>
@@ -3146,6 +3223,11 @@
           <t>COLUMN MAPPING — Map TFL table columns to treatment arms</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="73" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="68" t="inlineStr">
@@ -3153,6 +3235,11 @@
           <t>Define how each TFL's table columns map to treatment arms. If left empty, the validator falls back to substring matching on column headers.</t>
         </is>
       </c>
+      <c r="B2" s="72" t="n"/>
+      <c r="C2" s="72" t="n"/>
+      <c r="D2" s="72" t="n"/>
+      <c r="E2" s="72" t="n"/>
+      <c r="F2" s="73" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="69" t="inlineStr">
@@ -3371,6 +3458,11 @@
           <t>VARIABLE MAPPING — Override ADaM variable names and define validation variables</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="72" t="n"/>
+      <c r="E1" s="72" t="n"/>
+      <c r="F1" s="73" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="68" t="inlineStr">
@@ -3378,6 +3470,11 @@
           <t>Define which variables to validate per TFL, and override ADaM variable/flag names if your study uses non-standard names. If left empty, CDISC defaults are used.</t>
         </is>
       </c>
+      <c r="B2" s="72" t="n"/>
+      <c r="C2" s="72" t="n"/>
+      <c r="D2" s="72" t="n"/>
+      <c r="E2" s="72" t="n"/>
+      <c r="F2" s="73" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="69" t="inlineStr">
@@ -3721,6 +3818,11 @@
           <t>Variable Types: continuous, categorical, adam_flag, survival_param, survival_flag</t>
         </is>
       </c>
+      <c r="B16" s="72" t="n"/>
+      <c r="C16" s="72" t="n"/>
+      <c r="D16" s="72" t="n"/>
+      <c r="E16" s="72" t="n"/>
+      <c r="F16" s="73" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3754,6 +3856,9 @@
           <t>ROUNDING RULES — Configure decimal precision per statistic</t>
         </is>
       </c>
+      <c r="B1" s="72" t="n"/>
+      <c r="C1" s="72" t="n"/>
+      <c r="D1" s="73" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="68" t="inlineStr">
@@ -3761,6 +3866,9 @@
           <t>Set decimal places for comparisons. Use * as TFL ID for global defaults. TFL-specific entries override global. If empty, hardcoded defaults are used (Mean=1, SD=2, Percentage=1).</t>
         </is>
       </c>
+      <c r="B2" s="72" t="n"/>
+      <c r="C2" s="72" t="n"/>
+      <c r="D2" s="73" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="69" t="inlineStr">

</xml_diff>